<commit_message>
Add dataset_fix into Json folder
</commit_message>
<xml_diff>
--- a/Excel/ket_qua_nguyen_ban.xlsx
+++ b/Excel/ket_qua_nguyen_ban.xlsx
@@ -11938,12 +11938,6 @@
 $$</t>
   </si>
   <si>
-    <t>Xác định số họng tổng quát của dãy ($u_n$) được xác định bởi:
-$$
-u_1 = -2, \quad u_n = 3u_{n-1} - 1 \quad \forall n \ge 2.
-$$</t>
-  </si>
-  <si>
     <t>Xác định CTTQ của dãy $(u_n)$ được xác định: $u_1 = 2$; $u_n = 2u_{n-1} + 3n - 1$.</t>
   </si>
   <si>
@@ -15395,6 +15389,12 @@
 F(n + 2) = F(n + 1) + F(n), \forall n \in \mathbb{N}^*.
 $$
 Trong đó $F_1 = 1, F_2 = 1$. Các số $F(n)$ được gọi là các số Fibonacci. Trong các bài toán sau đây, $F(n)$ dùng để kí hiệu số Fibonacci thứ $n$.</t>
+  </si>
+  <si>
+    <t>Xác định số hạng tổng quát của dãy ($u_n$) được xác định bởi:
+$$
+u_1 = -2, \quad u_n = 3u_{n-1} - 1 \quad \forall n \ge 2.
+$$</t>
   </si>
 </sst>
 </file>
@@ -16188,7 +16188,7 @@
         <v>520</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
@@ -16196,10 +16196,10 @@
         <v>39</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>1500</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>1501</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>1502</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
@@ -16573,7 +16573,7 @@
         <v>1171</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>1499</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
@@ -16988,10 +16988,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C110" s="2" t="s">
         <v>1540</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>1541</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
@@ -17274,10 +17274,10 @@
         <v>137</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
@@ -17516,10 +17516,10 @@
         <v>159</v>
       </c>
       <c r="B158" s="2" t="s">
+        <v>1537</v>
+      </c>
+      <c r="C158" s="2" t="s">
         <v>1538</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>1539</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
@@ -17626,7 +17626,7 @@
         <v>169</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="C168" t="s">
         <v>887</v>
@@ -17761,7 +17761,7 @@
         <v>650</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>1535</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.35">
@@ -17849,7 +17849,7 @@
         <v>1177</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.35">
@@ -17860,7 +17860,7 @@
         <v>1178</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>1533</v>
+        <v>1532</v>
       </c>
       <c r="D189" s="3"/>
     </row>
@@ -17872,7 +17872,7 @@
         <v>1179</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>1531</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.35">
@@ -17883,7 +17883,7 @@
         <v>1180</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.35">
@@ -17891,10 +17891,10 @@
         <v>193</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.35">
@@ -17905,7 +17905,7 @@
         <v>1181</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>1527</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.35">
@@ -17916,7 +17916,7 @@
         <v>1182</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>1526</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.35">
@@ -17927,7 +17927,7 @@
         <v>1183</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>1524</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.35">
@@ -17938,7 +17938,7 @@
         <v>1184</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>1525</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.35">
@@ -17949,7 +17949,7 @@
         <v>1185</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="D197" s="3"/>
     </row>
@@ -17961,10 +17961,10 @@
         <v>1186</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.35">
@@ -17975,7 +17975,7 @@
         <v>1187</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>1523</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.35">
@@ -17986,7 +17986,7 @@
         <v>1188</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>1516</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.35">
@@ -17994,10 +17994,10 @@
         <v>202</v>
       </c>
       <c r="B201" s="2" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C201" s="2" t="s">
         <v>1514</v>
-      </c>
-      <c r="C201" s="2" t="s">
-        <v>1515</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.35">
@@ -18008,7 +18008,7 @@
         <v>1189</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>1530</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.35">
@@ -18019,7 +18019,7 @@
         <v>1190</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>1517</v>
+        <v>1516</v>
       </c>
       <c r="D203" s="3"/>
     </row>
@@ -18031,7 +18031,7 @@
         <v>1191</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>1518</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.35">
@@ -18042,10 +18042,10 @@
         <v>1192</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.35">
@@ -18177,7 +18177,7 @@
         <v>1203</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.35">
@@ -18691,10 +18691,10 @@
         <v>265</v>
       </c>
       <c r="B264" s="2" t="s">
+        <v>1511</v>
+      </c>
+      <c r="C264" s="2" t="s">
         <v>1512</v>
-      </c>
-      <c r="C264" s="2" t="s">
-        <v>1513</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.35">
@@ -18724,7 +18724,7 @@
         <v>268</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>1229</v>
+        <v>1541</v>
       </c>
       <c r="C267" t="s">
         <v>965</v>
@@ -18735,7 +18735,7 @@
         <v>269</v>
       </c>
       <c r="B268" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="C268" t="s">
         <v>966</v>
@@ -18746,7 +18746,7 @@
         <v>270</v>
       </c>
       <c r="B269" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="C269" s="2" t="s">
         <v>967</v>
@@ -18757,7 +18757,7 @@
         <v>271</v>
       </c>
       <c r="B270" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="C270" t="s">
         <v>968</v>
@@ -18768,7 +18768,7 @@
         <v>272</v>
       </c>
       <c r="B271" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="C271" t="s">
         <v>969</v>
@@ -18779,7 +18779,7 @@
         <v>273</v>
       </c>
       <c r="B272" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
       <c r="C272" t="s">
         <v>970</v>
@@ -18790,7 +18790,7 @@
         <v>274</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="C273" t="s">
         <v>971</v>
@@ -18801,7 +18801,7 @@
         <v>275</v>
       </c>
       <c r="B274" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="C274" t="s">
         <v>972</v>
@@ -18812,7 +18812,7 @@
         <v>276</v>
       </c>
       <c r="B275" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="C275" t="s">
         <v>973</v>
@@ -18823,7 +18823,7 @@
         <v>277</v>
       </c>
       <c r="B276" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="C276" t="s">
         <v>974</v>
@@ -18834,7 +18834,7 @@
         <v>278</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="C277" t="s">
         <v>975</v>
@@ -18845,7 +18845,7 @@
         <v>279</v>
       </c>
       <c r="B278" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="C278" t="s">
         <v>976</v>
@@ -18856,7 +18856,7 @@
         <v>280</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="C279" t="s">
         <v>977</v>
@@ -18867,7 +18867,7 @@
         <v>281</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="C280" t="s">
         <v>978</v>
@@ -18878,7 +18878,7 @@
         <v>282</v>
       </c>
       <c r="B281" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="C281" t="s">
         <v>979</v>
@@ -18889,7 +18889,7 @@
         <v>283</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="C282" t="s">
         <v>980</v>
@@ -18900,7 +18900,7 @@
         <v>284</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="C283" t="s">
         <v>981</v>
@@ -18911,7 +18911,7 @@
         <v>285</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="C284" t="s">
         <v>982</v>
@@ -18922,7 +18922,7 @@
         <v>286</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="C285" t="s">
         <v>983</v>
@@ -18933,7 +18933,7 @@
         <v>287</v>
       </c>
       <c r="B286" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="C286" t="s">
         <v>984</v>
@@ -18944,7 +18944,7 @@
         <v>288</v>
       </c>
       <c r="B287" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="C287" t="s">
         <v>985</v>
@@ -18955,7 +18955,7 @@
         <v>289</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="C288" t="s">
         <v>986</v>
@@ -18966,7 +18966,7 @@
         <v>290</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="C289" t="s">
         <v>987</v>
@@ -18977,7 +18977,7 @@
         <v>291</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="C290" t="s">
         <v>988</v>
@@ -18988,7 +18988,7 @@
         <v>292</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="C291" t="s">
         <v>989</v>
@@ -18999,7 +18999,7 @@
         <v>293</v>
       </c>
       <c r="B292" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="C292" t="s">
         <v>990</v>
@@ -19010,7 +19010,7 @@
         <v>294</v>
       </c>
       <c r="B293" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="C293" t="s">
         <v>991</v>
@@ -19021,7 +19021,7 @@
         <v>295</v>
       </c>
       <c r="B294" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="C294" t="s">
         <v>992</v>
@@ -19032,7 +19032,7 @@
         <v>296</v>
       </c>
       <c r="B295" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="C295" t="s">
         <v>993</v>
@@ -19043,7 +19043,7 @@
         <v>297</v>
       </c>
       <c r="B296" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C296" t="s">
         <v>994</v>
@@ -19054,7 +19054,7 @@
         <v>298</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="C297" t="s">
         <v>995</v>
@@ -19065,7 +19065,7 @@
         <v>299</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="C298" t="s">
         <v>996</v>
@@ -19076,7 +19076,7 @@
         <v>300</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="C299" t="s">
         <v>997</v>
@@ -19087,7 +19087,7 @@
         <v>301</v>
       </c>
       <c r="B300" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="C300" t="s">
         <v>998</v>
@@ -19098,7 +19098,7 @@
         <v>302</v>
       </c>
       <c r="B301" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="C301" t="s">
         <v>999</v>
@@ -19109,7 +19109,7 @@
         <v>303</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="C302" t="s">
         <v>1000</v>
@@ -19120,7 +19120,7 @@
         <v>304</v>
       </c>
       <c r="B303" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="C303" t="s">
         <v>1001</v>
@@ -19131,7 +19131,7 @@
         <v>305</v>
       </c>
       <c r="B304" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="C304" t="s">
         <v>1002</v>
@@ -19142,7 +19142,7 @@
         <v>306</v>
       </c>
       <c r="B305" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="C305" t="s">
         <v>1003</v>
@@ -19153,7 +19153,7 @@
         <v>307</v>
       </c>
       <c r="B306" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="C306" t="s">
         <v>1004</v>
@@ -19164,7 +19164,7 @@
         <v>308</v>
       </c>
       <c r="B307" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="C307" t="s">
         <v>1005</v>
@@ -19175,7 +19175,7 @@
         <v>309</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
       <c r="C308" t="s">
         <v>1006</v>
@@ -19186,7 +19186,7 @@
         <v>310</v>
       </c>
       <c r="B309" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="C309" t="s">
         <v>1007</v>
@@ -19197,7 +19197,7 @@
         <v>311</v>
       </c>
       <c r="B310" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="C310" t="s">
         <v>1008</v>
@@ -19263,7 +19263,7 @@
         <v>317</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="C316" t="s">
         <v>1014</v>
@@ -19318,7 +19318,7 @@
         <v>322</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C321" t="s">
         <v>1019</v>
@@ -19332,7 +19332,7 @@
         <v>691</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.35">
@@ -19384,7 +19384,7 @@
         <v>328</v>
       </c>
       <c r="B327" s="2" t="s">
-        <v>1500</v>
+        <v>1499</v>
       </c>
       <c r="C327" t="s">
         <v>1024</v>
@@ -19648,7 +19648,7 @@
         <v>352</v>
       </c>
       <c r="B351" s="2" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
       <c r="C351" t="s">
         <v>1048</v>
@@ -19714,7 +19714,7 @@
         <v>358</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="C357" t="s">
         <v>1054</v>
@@ -19725,7 +19725,7 @@
         <v>359</v>
       </c>
       <c r="B358" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="C358" t="s">
         <v>1055</v>
@@ -19769,7 +19769,7 @@
         <v>363</v>
       </c>
       <c r="B362" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="C362" t="s">
         <v>1059</v>
@@ -19791,7 +19791,7 @@
         <v>365</v>
       </c>
       <c r="B364" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="C364" t="s">
         <v>1061</v>
@@ -19802,7 +19802,7 @@
         <v>366</v>
       </c>
       <c r="B365" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="C365" t="s">
         <v>1062</v>
@@ -19813,7 +19813,7 @@
         <v>367</v>
       </c>
       <c r="B366" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="C366" t="s">
         <v>1063</v>
@@ -19824,7 +19824,7 @@
         <v>368</v>
       </c>
       <c r="B367" s="2" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="C367" t="s">
         <v>1064</v>
@@ -19835,7 +19835,7 @@
         <v>369</v>
       </c>
       <c r="B368" s="2" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="C368" t="s">
         <v>1065</v>
@@ -19846,7 +19846,7 @@
         <v>370</v>
       </c>
       <c r="B369" s="2" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="C369" t="s">
         <v>1066</v>
@@ -19857,7 +19857,7 @@
         <v>371</v>
       </c>
       <c r="B370" s="2" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="C370" t="s">
         <v>1067</v>
@@ -19868,7 +19868,7 @@
         <v>372</v>
       </c>
       <c r="B371" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="C371" t="s">
         <v>1068</v>
@@ -19879,7 +19879,7 @@
         <v>373</v>
       </c>
       <c r="B372" s="2" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C372" t="s">
         <v>1069</v>
@@ -19890,7 +19890,7 @@
         <v>374</v>
       </c>
       <c r="B373" s="2" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="C373" t="s">
         <v>1070</v>
@@ -19901,7 +19901,7 @@
         <v>375</v>
       </c>
       <c r="B374" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="C374" t="s">
         <v>1071</v>
@@ -19912,7 +19912,7 @@
         <v>376</v>
       </c>
       <c r="B375" s="2" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="C375" t="s">
         <v>1072</v>
@@ -19923,7 +19923,7 @@
         <v>377</v>
       </c>
       <c r="B376" s="2" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="C376" t="s">
         <v>1073</v>
@@ -19934,7 +19934,7 @@
         <v>378</v>
       </c>
       <c r="B377" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="C377" t="s">
         <v>1074</v>
@@ -19945,7 +19945,7 @@
         <v>379</v>
       </c>
       <c r="B378" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="C378" t="s">
         <v>1075</v>
@@ -19956,7 +19956,7 @@
         <v>380</v>
       </c>
       <c r="B379" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="C379" t="s">
         <v>1076</v>
@@ -19967,7 +19967,7 @@
         <v>381</v>
       </c>
       <c r="B380" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="C380" t="s">
         <v>1077</v>
@@ -19978,7 +19978,7 @@
         <v>382</v>
       </c>
       <c r="B381" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="C381" t="s">
         <v>1078</v>
@@ -19989,7 +19989,7 @@
         <v>383</v>
       </c>
       <c r="B382" s="2" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="C382" t="s">
         <v>1079</v>
@@ -20000,7 +20000,7 @@
         <v>384</v>
       </c>
       <c r="B383" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="C383" t="s">
         <v>1080</v>
@@ -20011,7 +20011,7 @@
         <v>385</v>
       </c>
       <c r="B384" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="C384" t="s">
         <v>1081</v>
@@ -20022,7 +20022,7 @@
         <v>386</v>
       </c>
       <c r="B385" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C385" t="s">
         <v>1082</v>
@@ -20033,7 +20033,7 @@
         <v>387</v>
       </c>
       <c r="B386" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="C386" t="s">
         <v>1083</v>
@@ -20044,7 +20044,7 @@
         <v>388</v>
       </c>
       <c r="B387" s="2" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="C387" t="s">
         <v>1084</v>
@@ -20055,7 +20055,7 @@
         <v>389</v>
       </c>
       <c r="B388" s="2" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="C388" t="s">
         <v>1085</v>
@@ -20066,7 +20066,7 @@
         <v>390</v>
       </c>
       <c r="B389" s="2" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="C389" t="s">
         <v>1086</v>
@@ -20077,7 +20077,7 @@
         <v>391</v>
       </c>
       <c r="B390" s="2" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="C390" t="s">
         <v>1087</v>
@@ -20088,7 +20088,7 @@
         <v>392</v>
       </c>
       <c r="B391" s="2" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="C391" t="s">
         <v>1088</v>
@@ -20099,7 +20099,7 @@
         <v>393</v>
       </c>
       <c r="B392" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="C392" t="s">
         <v>1089</v>
@@ -20110,7 +20110,7 @@
         <v>394</v>
       </c>
       <c r="B393" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="C393" t="s">
         <v>1090</v>
@@ -20121,7 +20121,7 @@
         <v>395</v>
       </c>
       <c r="B394" s="2" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="C394" t="s">
         <v>1091</v>
@@ -20132,7 +20132,7 @@
         <v>396</v>
       </c>
       <c r="B395" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="C395" t="s">
         <v>1092</v>
@@ -20143,7 +20143,7 @@
         <v>397</v>
       </c>
       <c r="B396" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="C396" t="s">
         <v>1093</v>
@@ -20154,7 +20154,7 @@
         <v>398</v>
       </c>
       <c r="B397" s="2" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="C397" t="s">
         <v>1094</v>
@@ -20165,7 +20165,7 @@
         <v>399</v>
       </c>
       <c r="B398" s="2" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="C398" t="s">
         <v>1095</v>
@@ -20176,7 +20176,7 @@
         <v>400</v>
       </c>
       <c r="B399" s="2" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="C399" t="s">
         <v>1096</v>
@@ -20187,7 +20187,7 @@
         <v>401</v>
       </c>
       <c r="B400" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="C400" t="s">
         <v>1097</v>
@@ -20198,7 +20198,7 @@
         <v>402</v>
       </c>
       <c r="B401" s="2" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="C401" t="s">
         <v>1098</v>
@@ -20209,7 +20209,7 @@
         <v>403</v>
       </c>
       <c r="B402" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="C402" t="s">
         <v>1099</v>
@@ -20220,7 +20220,7 @@
         <v>404</v>
       </c>
       <c r="B403" s="2" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="C403" t="s">
         <v>1100</v>
@@ -20231,7 +20231,7 @@
         <v>405</v>
       </c>
       <c r="B404" s="2" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="C404" t="s">
         <v>1101</v>
@@ -20242,10 +20242,10 @@
         <v>406</v>
       </c>
       <c r="B405" s="2" t="s">
+        <v>1318</v>
+      </c>
+      <c r="C405" s="2" t="s">
         <v>1319</v>
-      </c>
-      <c r="C405" s="2" t="s">
-        <v>1320</v>
       </c>
     </row>
     <row r="406" spans="1:3" x14ac:dyDescent="0.35">
@@ -20253,7 +20253,7 @@
         <v>407</v>
       </c>
       <c r="B406" s="2" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="C406" t="s">
         <v>1102</v>
@@ -20264,7 +20264,7 @@
         <v>408</v>
       </c>
       <c r="B407" s="2" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="C407" t="s">
         <v>1103</v>
@@ -20275,7 +20275,7 @@
         <v>409</v>
       </c>
       <c r="B408" s="2" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="C408" t="s">
         <v>1104</v>
@@ -20286,7 +20286,7 @@
         <v>410</v>
       </c>
       <c r="B409" s="2" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="C409" t="s">
         <v>1105</v>
@@ -20297,7 +20297,7 @@
         <v>411</v>
       </c>
       <c r="B410" s="2" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="C410" t="s">
         <v>1106</v>
@@ -20308,7 +20308,7 @@
         <v>412</v>
       </c>
       <c r="B411" s="2" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="C411" t="s">
         <v>1107</v>
@@ -20319,7 +20319,7 @@
         <v>413</v>
       </c>
       <c r="B412" s="2" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="C412" t="s">
         <v>1108</v>
@@ -20330,7 +20330,7 @@
         <v>414</v>
       </c>
       <c r="B413" s="2" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="C413" t="s">
         <v>1109</v>
@@ -20341,7 +20341,7 @@
         <v>415</v>
       </c>
       <c r="B414" s="2" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="C414" t="s">
         <v>1110</v>
@@ -20352,7 +20352,7 @@
         <v>416</v>
       </c>
       <c r="B415" s="2" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="C415" t="s">
         <v>1111</v>
@@ -20363,7 +20363,7 @@
         <v>417</v>
       </c>
       <c r="B416" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="C416" t="s">
         <v>1112</v>
@@ -20374,7 +20374,7 @@
         <v>418</v>
       </c>
       <c r="B417" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="C417" t="s">
         <v>1113</v>
@@ -20385,7 +20385,7 @@
         <v>419</v>
       </c>
       <c r="B418" s="2" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="C418" t="s">
         <v>1114</v>
@@ -20396,7 +20396,7 @@
         <v>420</v>
       </c>
       <c r="B419" s="2" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="C419" t="s">
         <v>1115</v>
@@ -20407,7 +20407,7 @@
         <v>421</v>
       </c>
       <c r="B420" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="C420" t="s">
         <v>1116</v>
@@ -20418,7 +20418,7 @@
         <v>422</v>
       </c>
       <c r="B421" s="2" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="C421" t="s">
         <v>1117</v>
@@ -20429,7 +20429,7 @@
         <v>423</v>
       </c>
       <c r="B422" s="2" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="C422" t="s">
         <v>1118</v>
@@ -20440,7 +20440,7 @@
         <v>424</v>
       </c>
       <c r="B423" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="C423" t="s">
         <v>1119</v>
@@ -20451,7 +20451,7 @@
         <v>425</v>
       </c>
       <c r="B424" s="2" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="C424" t="s">
         <v>1120</v>
@@ -20462,7 +20462,7 @@
         <v>426</v>
       </c>
       <c r="B425" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="C425" t="s">
         <v>1121</v>
@@ -20473,7 +20473,7 @@
         <v>427</v>
       </c>
       <c r="B426" s="2" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="C426" t="s">
         <v>1122</v>
@@ -20484,7 +20484,7 @@
         <v>428</v>
       </c>
       <c r="B427" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
       <c r="C427" t="s">
         <v>1123</v>
@@ -20495,7 +20495,7 @@
         <v>429</v>
       </c>
       <c r="B428" s="2" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="C428" t="s">
         <v>1124</v>
@@ -20506,7 +20506,7 @@
         <v>430</v>
       </c>
       <c r="B429" s="2" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="C429" t="s">
         <v>1125</v>
@@ -20517,7 +20517,7 @@
         <v>431</v>
       </c>
       <c r="B430" s="2" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="C430" t="s">
         <v>1126</v>
@@ -20528,7 +20528,7 @@
         <v>432</v>
       </c>
       <c r="B431" s="2" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="C431" t="s">
         <v>1127</v>
@@ -20539,7 +20539,7 @@
         <v>433</v>
       </c>
       <c r="B432" s="2" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="C432" t="s">
         <v>1128</v>
@@ -20550,7 +20550,7 @@
         <v>434</v>
       </c>
       <c r="B433" s="2" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="C433" t="s">
         <v>1129</v>
@@ -20561,7 +20561,7 @@
         <v>435</v>
       </c>
       <c r="B434" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="C434" s="2" t="s">
         <v>1130</v>
@@ -20572,7 +20572,7 @@
         <v>436</v>
       </c>
       <c r="B435" s="2" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="C435" t="s">
         <v>1131</v>
@@ -20583,7 +20583,7 @@
         <v>437</v>
       </c>
       <c r="B436" s="2" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="C436" t="s">
         <v>1132</v>
@@ -20594,10 +20594,10 @@
         <v>438</v>
       </c>
       <c r="B437" s="2" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="C437" s="2" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="438" spans="1:3" x14ac:dyDescent="0.35">
@@ -20605,7 +20605,7 @@
         <v>439</v>
       </c>
       <c r="B438" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="C438" t="s">
         <v>1133</v>
@@ -20616,7 +20616,7 @@
         <v>440</v>
       </c>
       <c r="B439" s="2" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="C439" t="s">
         <v>1134</v>
@@ -20627,7 +20627,7 @@
         <v>441</v>
       </c>
       <c r="B440" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="C440" t="s">
         <v>1135</v>
@@ -20638,7 +20638,7 @@
         <v>442</v>
       </c>
       <c r="B441" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="C441" t="s">
         <v>1136</v>
@@ -20649,7 +20649,7 @@
         <v>443</v>
       </c>
       <c r="B442" s="2" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="C442" t="s">
         <v>1137</v>
@@ -20660,7 +20660,7 @@
         <v>444</v>
       </c>
       <c r="B443" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="C443" t="s">
         <v>1138</v>
@@ -20671,7 +20671,7 @@
         <v>445</v>
       </c>
       <c r="B444" s="2" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="C444" t="s">
         <v>1139</v>
@@ -20682,7 +20682,7 @@
         <v>446</v>
       </c>
       <c r="B445" s="2" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="C445" t="s">
         <v>1140</v>
@@ -20693,7 +20693,7 @@
         <v>447</v>
       </c>
       <c r="B446" s="2" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="C446" t="s">
         <v>1141</v>
@@ -20704,7 +20704,7 @@
         <v>448</v>
       </c>
       <c r="B447" s="2" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="C447" t="s">
         <v>1142</v>
@@ -20715,7 +20715,7 @@
         <v>449</v>
       </c>
       <c r="B448" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="C448" t="s">
         <v>1143</v>
@@ -20726,7 +20726,7 @@
         <v>450</v>
       </c>
       <c r="B449" s="2" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="C449" t="s">
         <v>1144</v>
@@ -20737,7 +20737,7 @@
         <v>451</v>
       </c>
       <c r="B450" s="2" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="C450" t="s">
         <v>1145</v>
@@ -20748,7 +20748,7 @@
         <v>452</v>
       </c>
       <c r="B451" s="2" t="s">
-        <v>1366</v>
+        <v>1365</v>
       </c>
       <c r="C451" t="s">
         <v>1146</v>
@@ -20759,7 +20759,7 @@
         <v>453</v>
       </c>
       <c r="B452" s="2" t="s">
-        <v>1367</v>
+        <v>1366</v>
       </c>
       <c r="C452" t="s">
         <v>1147</v>
@@ -20770,7 +20770,7 @@
         <v>454</v>
       </c>
       <c r="B453" s="2" t="s">
-        <v>1368</v>
+        <v>1367</v>
       </c>
       <c r="C453" t="s">
         <v>1148</v>
@@ -20781,7 +20781,7 @@
         <v>455</v>
       </c>
       <c r="B454" s="2" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="C454" t="s">
         <v>1149</v>
@@ -20792,10 +20792,10 @@
         <v>456</v>
       </c>
       <c r="B455" s="2" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
       <c r="C455" s="2" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="456" spans="1:3" x14ac:dyDescent="0.35">
@@ -20803,7 +20803,7 @@
         <v>457</v>
       </c>
       <c r="B456" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="C456" t="s">
         <v>1150</v>
@@ -20814,7 +20814,7 @@
         <v>458</v>
       </c>
       <c r="B457" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
       <c r="C457" t="s">
         <v>1151</v>
@@ -20825,7 +20825,7 @@
         <v>459</v>
       </c>
       <c r="B458" s="2" t="s">
-        <v>1373</v>
+        <v>1372</v>
       </c>
       <c r="C458" t="s">
         <v>1152</v>
@@ -20836,7 +20836,7 @@
         <v>460</v>
       </c>
       <c r="B459" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
       <c r="C459" t="s">
         <v>1153</v>
@@ -20847,7 +20847,7 @@
         <v>461</v>
       </c>
       <c r="B460" s="2" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="C460" t="s">
         <v>1154</v>
@@ -20858,7 +20858,7 @@
         <v>462</v>
       </c>
       <c r="B461" t="s">
-        <v>1376</v>
+        <v>1375</v>
       </c>
       <c r="C461" t="s">
         <v>1155</v>
@@ -20869,7 +20869,7 @@
         <v>463</v>
       </c>
       <c r="B462" t="s">
-        <v>1377</v>
+        <v>1376</v>
       </c>
       <c r="C462" t="s">
         <v>1156</v>
@@ -20880,7 +20880,7 @@
         <v>464</v>
       </c>
       <c r="B463" s="2" t="s">
-        <v>1378</v>
+        <v>1377</v>
       </c>
       <c r="C463" t="s">
         <v>1157</v>
@@ -20891,7 +20891,7 @@
         <v>465</v>
       </c>
       <c r="B464" s="2" t="s">
-        <v>1379</v>
+        <v>1378</v>
       </c>
       <c r="C464" t="s">
         <v>1158</v>
@@ -20902,7 +20902,7 @@
         <v>466</v>
       </c>
       <c r="B465" s="2" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="C465" t="s">
         <v>1159</v>
@@ -20913,7 +20913,7 @@
         <v>467</v>
       </c>
       <c r="B466" s="2" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
       <c r="C466" t="s">
         <v>1160</v>
@@ -20924,7 +20924,7 @@
         <v>468</v>
       </c>
       <c r="B467" s="2" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
       <c r="C467" t="s">
         <v>1161</v>
@@ -20935,7 +20935,7 @@
         <v>469</v>
       </c>
       <c r="B468" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
       <c r="C468" t="s">
         <v>1162</v>
@@ -20946,7 +20946,7 @@
         <v>470</v>
       </c>
       <c r="B469" s="2" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
       <c r="C469" t="s">
         <v>1163</v>
@@ -20957,7 +20957,7 @@
         <v>471</v>
       </c>
       <c r="B470" s="2" t="s">
-        <v>1385</v>
+        <v>1384</v>
       </c>
       <c r="C470" t="s">
         <v>1164</v>
@@ -20968,7 +20968,7 @@
         <v>472</v>
       </c>
       <c r="B471" s="2" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="C471" t="s">
         <v>1165</v>
@@ -20979,7 +20979,7 @@
         <v>473</v>
       </c>
       <c r="B472" s="2" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="C472" t="s">
         <v>1166</v>
@@ -20990,7 +20990,7 @@
         <v>474</v>
       </c>
       <c r="B473" s="2" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="C473" t="s">
         <v>1167</v>
@@ -21001,7 +21001,7 @@
         <v>475</v>
       </c>
       <c r="B474" s="2" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
       <c r="C474" t="s">
         <v>1168</v>
@@ -21012,10 +21012,10 @@
         <v>476</v>
       </c>
       <c r="B475" t="s">
+        <v>1389</v>
+      </c>
+      <c r="C475" t="s">
         <v>1390</v>
-      </c>
-      <c r="C475" t="s">
-        <v>1391</v>
       </c>
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.35">
@@ -21023,10 +21023,10 @@
         <v>477</v>
       </c>
       <c r="B476" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C476" t="s">
         <v>1392</v>
-      </c>
-      <c r="C476" t="s">
-        <v>1393</v>
       </c>
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.35">
@@ -21034,10 +21034,10 @@
         <v>478</v>
       </c>
       <c r="B477" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C477" t="s">
         <v>1394</v>
-      </c>
-      <c r="C477" t="s">
-        <v>1395</v>
       </c>
     </row>
     <row r="478" spans="1:3" x14ac:dyDescent="0.35">
@@ -21045,10 +21045,10 @@
         <v>479</v>
       </c>
       <c r="B478" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C478" t="s">
         <v>1396</v>
-      </c>
-      <c r="C478" t="s">
-        <v>1397</v>
       </c>
     </row>
     <row r="479" spans="1:3" x14ac:dyDescent="0.35">
@@ -21056,10 +21056,10 @@
         <v>480</v>
       </c>
       <c r="B479" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C479" t="s">
         <v>1398</v>
-      </c>
-      <c r="C479" t="s">
-        <v>1399</v>
       </c>
     </row>
     <row r="480" spans="1:3" x14ac:dyDescent="0.35">
@@ -21067,10 +21067,10 @@
         <v>481</v>
       </c>
       <c r="B480" t="s">
+        <v>1399</v>
+      </c>
+      <c r="C480" t="s">
         <v>1400</v>
-      </c>
-      <c r="C480" t="s">
-        <v>1401</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.35">
@@ -21078,10 +21078,10 @@
         <v>482</v>
       </c>
       <c r="B481" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C481" t="s">
         <v>1402</v>
-      </c>
-      <c r="C481" t="s">
-        <v>1403</v>
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.35">
@@ -21089,10 +21089,10 @@
         <v>483</v>
       </c>
       <c r="B482" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C482" t="s">
         <v>1404</v>
-      </c>
-      <c r="C482" t="s">
-        <v>1405</v>
       </c>
     </row>
     <row r="483" spans="1:3" x14ac:dyDescent="0.35">
@@ -21100,351 +21100,351 @@
         <v>484</v>
       </c>
       <c r="B483" t="s">
+        <v>1405</v>
+      </c>
+      <c r="C483" t="s">
         <v>1406</v>
-      </c>
-      <c r="C483" t="s">
-        <v>1407</v>
       </c>
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A484" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
       <c r="B484" t="s">
+        <v>1407</v>
+      </c>
+      <c r="C484" t="s">
         <v>1408</v>
-      </c>
-      <c r="C484" t="s">
-        <v>1409</v>
       </c>
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A485" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="B485" s="2" t="s">
+        <v>1409</v>
+      </c>
+      <c r="C485" t="s">
         <v>1410</v>
-      </c>
-      <c r="C485" t="s">
-        <v>1411</v>
       </c>
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
       <c r="B486" s="2" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
       <c r="C486" s="2" t="s">
-        <v>1412</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A487" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="B487" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C487" t="s">
         <v>1413</v>
-      </c>
-      <c r="C487" t="s">
-        <v>1414</v>
       </c>
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A488" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="B488" t="s">
+        <v>1414</v>
+      </c>
+      <c r="C488" t="s">
         <v>1415</v>
-      </c>
-      <c r="C488" t="s">
-        <v>1416</v>
       </c>
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A489" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
       <c r="B489" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C489" t="s">
         <v>1417</v>
-      </c>
-      <c r="C489" t="s">
-        <v>1418</v>
       </c>
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="B490" t="s">
+        <v>1418</v>
+      </c>
+      <c r="C490" t="s">
         <v>1419</v>
-      </c>
-      <c r="C490" t="s">
-        <v>1420</v>
       </c>
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="B491" t="s">
+        <v>1420</v>
+      </c>
+      <c r="C491" t="s">
         <v>1421</v>
-      </c>
-      <c r="C491" t="s">
-        <v>1422</v>
       </c>
     </row>
     <row r="492" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A492" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B492" t="s">
+        <v>1422</v>
+      </c>
+      <c r="C492" t="s">
         <v>1423</v>
-      </c>
-      <c r="C492" t="s">
-        <v>1424</v>
       </c>
     </row>
     <row r="493" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A493" t="s">
-        <v>1476</v>
+        <v>1475</v>
       </c>
       <c r="B493" t="s">
+        <v>1424</v>
+      </c>
+      <c r="C493" t="s">
         <v>1425</v>
-      </c>
-      <c r="C493" t="s">
-        <v>1426</v>
       </c>
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A494" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
       <c r="B494" t="s">
+        <v>1426</v>
+      </c>
+      <c r="C494" t="s">
         <v>1427</v>
-      </c>
-      <c r="C494" t="s">
-        <v>1428</v>
       </c>
     </row>
     <row r="495" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A495" t="s">
-        <v>1478</v>
+        <v>1477</v>
       </c>
       <c r="B495" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C495" t="s">
         <v>1429</v>
-      </c>
-      <c r="C495" t="s">
-        <v>1430</v>
       </c>
     </row>
     <row r="496" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A496" t="s">
-        <v>1479</v>
+        <v>1478</v>
       </c>
       <c r="B496" t="s">
+        <v>1430</v>
+      </c>
+      <c r="C496" t="s">
         <v>1431</v>
-      </c>
-      <c r="C496" t="s">
-        <v>1432</v>
       </c>
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A497" t="s">
-        <v>1480</v>
+        <v>1479</v>
       </c>
       <c r="B497" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C497" t="s">
         <v>1433</v>
-      </c>
-      <c r="C497" t="s">
-        <v>1434</v>
       </c>
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A498" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="B498" t="s">
+        <v>1434</v>
+      </c>
+      <c r="C498" t="s">
         <v>1435</v>
-      </c>
-      <c r="C498" t="s">
-        <v>1436</v>
       </c>
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="B499" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C499" t="s">
         <v>1437</v>
-      </c>
-      <c r="C499" t="s">
-        <v>1438</v>
       </c>
     </row>
     <row r="500" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A500" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
       <c r="B500" t="s">
+        <v>1438</v>
+      </c>
+      <c r="C500" t="s">
         <v>1439</v>
-      </c>
-      <c r="C500" t="s">
-        <v>1440</v>
       </c>
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A501" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
       <c r="B501" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C501" t="s">
         <v>1441</v>
-      </c>
-      <c r="C501" t="s">
-        <v>1442</v>
       </c>
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A502" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
       <c r="B502" t="s">
+        <v>1442</v>
+      </c>
+      <c r="C502" t="s">
         <v>1443</v>
-      </c>
-      <c r="C502" t="s">
-        <v>1444</v>
       </c>
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A503" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="B503" t="s">
+        <v>1444</v>
+      </c>
+      <c r="C503" t="s">
         <v>1445</v>
-      </c>
-      <c r="C503" t="s">
-        <v>1446</v>
       </c>
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A504" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
       <c r="B504" s="2" t="s">
-        <v>1510</v>
+        <v>1509</v>
       </c>
       <c r="C504" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A505" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
       <c r="B505" t="s">
+        <v>1447</v>
+      </c>
+      <c r="C505" t="s">
         <v>1448</v>
-      </c>
-      <c r="C505" t="s">
-        <v>1449</v>
       </c>
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A506" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
       <c r="B506" t="s">
+        <v>1449</v>
+      </c>
+      <c r="C506" t="s">
         <v>1450</v>
-      </c>
-      <c r="C506" t="s">
-        <v>1451</v>
       </c>
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A507" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
       <c r="B507" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C507" t="s">
         <v>1452</v>
-      </c>
-      <c r="C507" t="s">
-        <v>1453</v>
       </c>
     </row>
     <row r="508" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A508" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
       <c r="B508" t="s">
+        <v>1453</v>
+      </c>
+      <c r="C508" t="s">
         <v>1454</v>
-      </c>
-      <c r="C508" t="s">
-        <v>1455</v>
       </c>
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A509" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
       <c r="B509" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C509" t="s">
         <v>1456</v>
-      </c>
-      <c r="C509" t="s">
-        <v>1457</v>
       </c>
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A510" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
       <c r="B510" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C510" t="s">
         <v>1458</v>
-      </c>
-      <c r="C510" t="s">
-        <v>1459</v>
       </c>
     </row>
     <row r="511" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A511" t="s">
-        <v>1494</v>
+        <v>1493</v>
       </c>
       <c r="B511" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C511" t="s">
         <v>1460</v>
-      </c>
-      <c r="C511" t="s">
-        <v>1461</v>
       </c>
     </row>
     <row r="512" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A512" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="B512" t="s">
+        <v>1461</v>
+      </c>
+      <c r="C512" t="s">
         <v>1462</v>
-      </c>
-      <c r="C512" t="s">
-        <v>1463</v>
       </c>
     </row>
     <row r="513" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A513" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="B513" t="s">
+        <v>1463</v>
+      </c>
+      <c r="C513" t="s">
         <v>1464</v>
-      </c>
-      <c r="C513" t="s">
-        <v>1465</v>
       </c>
     </row>
     <row r="514" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A514" t="s">
-        <v>1497</v>
+        <v>1496</v>
       </c>
       <c r="B514" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="C514" s="2" t="s">
-        <v>1536</v>
+        <v>1535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>